<commit_message>
v.1.5.5: Language Settings - Fase 3
- data for spanish, english and valencian
- Language Settings finished
</commit_message>
<xml_diff>
--- a/data/memories/memory_01/locales/es/documents/archive/Contracts Registry.xlsx
+++ b/data/memories/memory_01/locales/es/documents/archive/Contracts Registry.xlsx
@@ -433,7 +433,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Contracts Registry</t>
+          <t>Registro de Contratos</t>
         </is>
       </c>
     </row>
@@ -445,7 +445,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Internal Archive</t>
+          <t>Archivo Interno</t>
         </is>
       </c>
     </row>
@@ -469,55 +469,55 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Archive Department</t>
+          <t>Departamento de Archivo</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Contract Registry Overview</t>
+          <t>Descripción general del registro de contratos</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>This registry contains a historical index of contracts stored in the company archive. The purpose of the document is to provide traceability between physical documents and digital references.</t>
+          <t>Este registro contiene un índice histórico de los contratos almacenados en el archivo de la empresa. El objetivo del documento es proporcionar trazabilidad entre documentos físicos y referencias digitales.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Registered Documents</t>
+          <t>Documentos registrados</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Referencia</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Categoría</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Year</t>
+          <t>Año</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Location</t>
+          <t>Ubicación</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Estado</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Supplier Agreement</t>
+          <t>Acuerdo de proveedor</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -539,12 +539,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Archive Cabinet A</t>
+          <t>Gabinete de archivo A</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Disponible</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Technology Services</t>
+          <t>Servicios Tecnológicos</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -566,12 +566,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Archive Cabinet B</t>
+          <t>Gabinete de archivo B</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Disponible</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Facilities Agreement</t>
+          <t>Acuerdo de instalaciones</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -593,12 +593,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Archive Cabinet C</t>
+          <t>Gabinete de archivo C</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Available</t>
+          <t>Disponible</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Operations Support</t>
+          <t>Soporte de operaciones</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Archive Cabinet G</t>
+          <t>Gabinete de archivo G</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Review Required</t>
+          <t>Revisión requerida</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Internal Services</t>
+          <t>Servicios Internos</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -647,68 +647,68 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Desconocido</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Verification Pending</t>
+          <t>Verificación pendiente</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Registry Observations</t>
+          <t>Observaciones del Registro</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Several older references were created before the current document classification system was introduced. These entries should remain unchanged until the archive migration is complete.</t>
+          <t>Se crearon varias referencias antiguas antes de que se introdujera el sistema de clasificación de documentos actual. Estas entradas deben permanecer sin cambios hasta que se complete la migración del archivo.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CTR-004 requires additional review because its location corresponds to a cabinet excluded from previous inventory reports.</t>
+          <t>CTR-004 requiere revisión adicional porque su ubicación corresponde a un gabinete excluido de informes de inventario anteriores.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Retention Policy</t>
+          <t>Política de retención</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>• Do not destroy historical contracts.</t>
+          <t>• No destruyas contratos históricos.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>• Preserve original identifiers.</t>
+          <t>• Conservar los identificadores originales.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>• Record all archive movements.</t>
+          <t>• Registre todos los movimientos del archivo.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>• Maintain access history.</t>
+          <t>• Mantener el historial de acceso.</t>
         </is>
       </c>
     </row>

</xml_diff>